<commit_message>
Enhancement: Support 'Github ID' column name and generate fallback emails for simplified student imports.
</commit_message>
<xml_diff>
--- a/backend/templates/student_import.xlsx
+++ b/backend/templates/student_import.xlsx
@@ -14,76 +14,28 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
-    <t>name</t>
+    <t>Name</t>
   </si>
   <si>
-    <t>email</t>
+    <t>Github ID</t>
   </si>
   <si>
-    <t>roll_number</t>
+    <t>Email</t>
   </si>
   <si>
-    <t>github</t>
+    <t>Roll Number</t>
   </si>
   <si>
-    <t>department</t>
-  </si>
-  <si>
-    <t>phone</t>
-  </si>
-  <si>
-    <t>leetcode_username</t>
-  </si>
-  <si>
-    <t>John Doe</t>
-  </si>
-  <si>
-    <t>Jane Smith</t>
-  </si>
-  <si>
-    <t>john@example.edu</t>
-  </si>
-  <si>
-    <t>jane@example.edu</t>
-  </si>
-  <si>
-    <t>2024CS01</t>
-  </si>
-  <si>
-    <t>2024CS02</t>
-  </si>
-  <si>
-    <t>https://github.com/johndoe</t>
-  </si>
-  <si>
-    <t>https://github.com/janesmith</t>
-  </si>
-  <si>
-    <t>Computer Science</t>
-  </si>
-  <si>
-    <t>Information Technology</t>
-  </si>
-  <si>
-    <t>1234567890</t>
-  </si>
-  <si>
-    <t>0987654321</t>
-  </si>
-  <si>
-    <t>johndoe_lc</t>
-  </si>
-  <si>
-    <t>janesmith_lc</t>
+    <t>Department</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -98,13 +50,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -139,22 +84,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="top"/>
-      <protection locked="0"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -447,10 +386,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -466,64 +405,8 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="D2" r:id="rId1"/>
-    <hyperlink ref="D3" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>